<commit_message>
Add sample S1A8 (SRR26147254) to annexes 3, 4, 7-11
The run was missing from the downloads. It was processed like the other
samples (pychopper -Q 9 -q 0.52 edlib, filtlong 1000-1700 pb, EMU 3.6.2),
and the annexes were regenerated with 89 samples: Pearson 0.9925 (family),
0.9862 (genus) and 0.9635 (species, 854 shared); PERMANOVA CS vs CSSwP
pseudo-F 0.421, p 0.642 (n = 88); annex 11 now compares 88 samples.
</commit_message>
<xml_diff>
--- a/Anexo_03_Estadisticas_pre_limpieza/Anexo_03_Estadisticas_pre_limpieza.xlsx
+++ b/Anexo_03_Estadisticas_pre_limpieza/Anexo_03_Estadisticas_pre_limpieza.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="2" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Estadísticas pre limpieza" sheetId="1" state="visible" r:id="rId1"/>
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:M98"/>
+  <dimension ref="A2:M99"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="13.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col width="13.5703125" customWidth="1" style="1" min="1" max="1"/>
@@ -1650,38 +1650,38 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>SRR26147265</t>
+          <t>SRR26147254</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>22233</v>
+        <v>21457</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>31604135</v>
+        <v>30682044</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>1421.5</v>
+        <v>1429.93</v>
       </c>
       <c r="G33" s="3" t="n">
         <v>75</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>4064</v>
+        <v>5060</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>1458</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>53.92</v>
+        <v>53.91</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>17.41</v>
+        <v>17.36</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>9.619999999999999</v>
+        <v>10.07</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>24.62</v>
+        <v>25.17</v>
       </c>
     </row>
     <row r="34">
@@ -1690,38 +1690,38 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>SRR26147276</t>
+          <t>SRR26147265</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>42222</v>
+        <v>22233</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>60294554</v>
+        <v>31604135</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>1428.04</v>
+        <v>1421.5</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>3077</v>
+        <v>4064</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>1458</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>53.87</v>
+        <v>53.92</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>17.36</v>
+        <v>17.41</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>8.630000000000001</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>25.71</v>
+        <v>24.62</v>
       </c>
     </row>
     <row r="35">
@@ -1730,38 +1730,38 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>SRR26147286</t>
+          <t>SRR26147276</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>14271</v>
+        <v>42222</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>20451980</v>
+        <v>60294554</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>1433.11</v>
+        <v>1428.04</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>4235</v>
+        <v>3077</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>1463</v>
+        <v>1458</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>56.05</v>
+        <v>53.87</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>17.12</v>
+        <v>17.36</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>10.27</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>23.41</v>
+        <v>25.71</v>
       </c>
     </row>
     <row r="36">
@@ -1770,38 +1770,38 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>SRR26147287</t>
+          <t>SRR26147286</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>20063</v>
+        <v>14271</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>29024181</v>
+        <v>20451980</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>1446.65</v>
+        <v>1433.11</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>4224</v>
+        <v>4235</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>1464</v>
+        <v>1463</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>55.82</v>
+        <v>56.05</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>17.17</v>
+        <v>17.12</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>9.68</v>
+        <v>10.27</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>24.15</v>
+        <v>23.41</v>
       </c>
     </row>
     <row r="37">
@@ -1810,38 +1810,38 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>SRR26147288</t>
+          <t>SRR26147287</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>28026</v>
+        <v>20063</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>40417934</v>
+        <v>29024181</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>1442.16</v>
+        <v>1446.65</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>3528</v>
+        <v>4224</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>1463</v>
+        <v>1464</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>55.92</v>
+        <v>55.82</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>17.08</v>
+        <v>17.17</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>10.3</v>
+        <v>9.68</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>23.9</v>
+        <v>24.15</v>
       </c>
     </row>
     <row r="38">
@@ -1850,38 +1850,38 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>SRR26147289</t>
+          <t>SRR26147288</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>33334</v>
+        <v>28026</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>48237676</v>
+        <v>40417934</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>1447.1</v>
+        <v>1442.16</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>5638</v>
+        <v>3528</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>1463</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>56.01</v>
+        <v>55.92</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>17.19</v>
+        <v>17.08</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>9.119999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>24.89</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="39">
@@ -1890,38 +1890,38 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>SRR26147290</t>
+          <t>SRR26147289</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>22108</v>
+        <v>33334</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>31969410</v>
+        <v>48237676</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>1446.06</v>
+        <v>1447.1</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>3904</v>
+        <v>5638</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>1464</v>
+        <v>1463</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>55.85</v>
+        <v>56.01</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>17.31</v>
+        <v>17.19</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>10.54</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>23.96</v>
+        <v>24.89</v>
       </c>
     </row>
     <row r="40">
@@ -1930,38 +1930,38 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>SRR26147292</t>
+          <t>SRR26147290</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>28388</v>
+        <v>22108</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>40837637</v>
+        <v>31969410</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>1438.55</v>
+        <v>1446.06</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>3946</v>
+        <v>3904</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>1464</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>55.89</v>
+        <v>55.85</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>17.25</v>
+        <v>17.31</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>9.81</v>
+        <v>10.54</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>24.24</v>
+        <v>23.96</v>
       </c>
     </row>
     <row r="41">
@@ -1970,38 +1970,38 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>SRR26147303</t>
+          <t>SRR26147292</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>16617</v>
+        <v>28388</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>23974117</v>
+        <v>40837637</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>1442.75</v>
+        <v>1438.55</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>3900</v>
+        <v>3946</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>1463</v>
+        <v>1464</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>56.1</v>
+        <v>55.89</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>17.22</v>
+        <v>17.25</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>10.38</v>
+        <v>9.81</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>23.91</v>
+        <v>24.24</v>
       </c>
     </row>
     <row r="42">
@@ -2010,38 +2010,38 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>SRR26147314</t>
+          <t>SRR26147303</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>38828</v>
+        <v>16617</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>55654270</v>
+        <v>23974117</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>1433.35</v>
+        <v>1442.75</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>4039</v>
+        <v>3900</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>1458</v>
+        <v>1463</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>54.51</v>
+        <v>56.1</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>17.32</v>
+        <v>17.22</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>9.91</v>
+        <v>10.38</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>24.89</v>
+        <v>23.91</v>
       </c>
     </row>
     <row r="43">
@@ -2050,38 +2050,38 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>SRR26147329</t>
+          <t>SRR26147314</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>19112</v>
+        <v>38828</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>27593762</v>
+        <v>55654270</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>1443.79</v>
+        <v>1433.35</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>4235</v>
+        <v>4039</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>1464</v>
+        <v>1458</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>55.65</v>
+        <v>54.51</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>17.15</v>
+        <v>17.32</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>10.53</v>
+        <v>9.91</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>23.98</v>
+        <v>24.89</v>
       </c>
     </row>
     <row r="44">
@@ -2090,38 +2090,38 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>SRR26147340</t>
+          <t>SRR26147329</t>
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>42838</v>
+        <v>19112</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>61882478</v>
+        <v>27593762</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>1444.57</v>
+        <v>1443.79</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>4536</v>
+        <v>4235</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>1462</v>
+        <v>1464</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>55.78</v>
+        <v>55.65</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>17.17</v>
+        <v>17.15</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>9.890000000000001</v>
+        <v>10.53</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>24.33</v>
+        <v>23.98</v>
       </c>
     </row>
     <row r="45">
@@ -2130,38 +2130,38 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>SRR26147351</t>
+          <t>SRR26147340</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>26016</v>
+        <v>42838</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>37500775</v>
+        <v>61882478</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>1441.45</v>
+        <v>1444.57</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>3620</v>
+        <v>4536</v>
       </c>
       <c r="I45" s="3" t="n">
         <v>1462</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>55.99</v>
+        <v>55.78</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>17.13</v>
+        <v>17.17</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>10.39</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>24.67</v>
+        <v>24.33</v>
       </c>
     </row>
     <row r="46">
@@ -2170,38 +2170,38 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>SRR26147365</t>
+          <t>SRR26147351</t>
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>16344</v>
+        <v>26016</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>23112638</v>
+        <v>37500775</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>1414.14</v>
+        <v>1441.45</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>3114</v>
+        <v>3620</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>1460</v>
+        <v>1462</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>53.94</v>
+        <v>55.99</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>17.46</v>
+        <v>17.13</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>9.470000000000001</v>
+        <v>10.39</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>24.35</v>
+        <v>24.67</v>
       </c>
     </row>
     <row r="47">
@@ -2210,38 +2210,38 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>SRR26147376</t>
+          <t>SRR26147365</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>42843</v>
+        <v>16344</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>61642735</v>
+        <v>23112638</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>1438.81</v>
+        <v>1414.14</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>3836</v>
+        <v>3114</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>1459</v>
+        <v>1460</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>53.96</v>
+        <v>53.94</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>17.29</v>
+        <v>17.46</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>9.890000000000001</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="M47" s="3" t="n">
-        <v>23.87</v>
+        <v>24.35</v>
       </c>
     </row>
     <row r="48">
@@ -2250,38 +2250,38 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>SRR26147387</t>
+          <t>SRR26147376</t>
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>40446</v>
+        <v>42843</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>58478733</v>
+        <v>61642735</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>1445.85</v>
+        <v>1438.81</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>110</v>
+        <v>76</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>3553</v>
+        <v>3836</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>1466</v>
+        <v>1459</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>55.72</v>
+        <v>53.96</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>17.2</v>
+        <v>17.29</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>9.970000000000001</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="M48" s="3" t="n">
-        <v>24.56</v>
+        <v>23.87</v>
       </c>
     </row>
     <row r="49">
@@ -2290,38 +2290,38 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>SRR26147388</t>
+          <t>SRR26147387</t>
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>27376</v>
+        <v>40446</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>39658991</v>
+        <v>58478733</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>1448.68</v>
+        <v>1445.85</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>81</v>
+        <v>110</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>4140</v>
+        <v>3553</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>1465</v>
+        <v>1466</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>55.59</v>
+        <v>55.72</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>17.22</v>
+        <v>17.2</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>9.08</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>24.29</v>
+        <v>24.56</v>
       </c>
     </row>
     <row r="50">
@@ -2330,38 +2330,38 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>SRR26147389</t>
+          <t>SRR26147388</t>
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>26136</v>
+        <v>27376</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>37827688</v>
+        <v>39658991</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>1447.34</v>
+        <v>1448.68</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>3781</v>
+        <v>4140</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>1466</v>
+        <v>1465</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>55.86</v>
+        <v>55.59</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>17.25</v>
+        <v>17.22</v>
       </c>
       <c r="L50" s="3" t="n">
-        <v>10.24</v>
+        <v>9.08</v>
       </c>
       <c r="M50" s="3" t="n">
-        <v>23.93</v>
+        <v>24.29</v>
       </c>
     </row>
     <row r="51">
@@ -2370,38 +2370,38 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>SRR26147390</t>
+          <t>SRR26147389</t>
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>31175</v>
+        <v>26136</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>45183903</v>
+        <v>37827688</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>1449.36</v>
+        <v>1447.34</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>4198</v>
+        <v>3781</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>1464</v>
+        <v>1466</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>56.05</v>
+        <v>55.86</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>17.15</v>
+        <v>17.25</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>10.23</v>
+        <v>10.24</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>23.95</v>
+        <v>23.93</v>
       </c>
     </row>
     <row r="52">
@@ -2410,38 +2410,38 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>SRR26147391</t>
+          <t>SRR26147390</t>
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>33527</v>
+        <v>31175</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>48035795</v>
+        <v>45183903</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>1432.75</v>
+        <v>1449.36</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>4199</v>
+        <v>4198</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>1458</v>
+        <v>1464</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>54.96</v>
+        <v>56.05</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>17.17</v>
+        <v>17.15</v>
       </c>
       <c r="L52" s="3" t="n">
-        <v>9.710000000000001</v>
+        <v>10.23</v>
       </c>
       <c r="M52" s="3" t="n">
-        <v>25.05</v>
+        <v>23.95</v>
       </c>
     </row>
     <row r="53">
@@ -2450,38 +2450,38 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>SRR26147392</t>
+          <t>SRR26147391</t>
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>19180</v>
+        <v>33527</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>27461423</v>
+        <v>48035795</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>1431.77</v>
+        <v>1432.75</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>3545</v>
+        <v>4199</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>1457</v>
+        <v>1458</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>55.03</v>
+        <v>54.96</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>17.28</v>
+        <v>17.17</v>
       </c>
       <c r="L53" s="3" t="n">
         <v>9.710000000000001</v>
       </c>
       <c r="M53" s="3" t="n">
-        <v>24.07</v>
+        <v>25.05</v>
       </c>
     </row>
     <row r="54">
@@ -2490,26 +2490,26 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>SRR26147393</t>
+          <t>SRR26147392</t>
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>14482</v>
+        <v>19180</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>20658852</v>
+        <v>27461423</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>1426.52</v>
+        <v>1431.77</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>2998</v>
+        <v>3545</v>
       </c>
       <c r="I54" s="3" t="n">
-        <v>1460</v>
+        <v>1457</v>
       </c>
       <c r="J54" s="3" t="n">
         <v>55.03</v>
@@ -2518,10 +2518,10 @@
         <v>17.28</v>
       </c>
       <c r="L54" s="3" t="n">
-        <v>10.62</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="M54" s="3" t="n">
-        <v>24.88</v>
+        <v>24.07</v>
       </c>
     </row>
     <row r="55">
@@ -2530,38 +2530,38 @@
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>SRR26147394</t>
+          <t>SRR26147393</t>
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>29279</v>
+        <v>14482</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>42142708</v>
+        <v>20658852</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>1439.35</v>
+        <v>1426.52</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>4275</v>
+        <v>2998</v>
       </c>
       <c r="I55" s="3" t="n">
-        <v>1463</v>
+        <v>1460</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>55.76</v>
+        <v>55.03</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>17.13</v>
+        <v>17.28</v>
       </c>
       <c r="L55" s="3" t="n">
-        <v>10.32</v>
+        <v>10.62</v>
       </c>
       <c r="M55" s="3" t="n">
-        <v>24.63</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="56">
@@ -2570,38 +2570,38 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>SRR26147395</t>
+          <t>SRR26147394</t>
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>23407</v>
+        <v>29279</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>33487460</v>
+        <v>42142708</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>1430.66</v>
+        <v>1439.35</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>4013</v>
+        <v>4275</v>
       </c>
       <c r="I56" s="3" t="n">
-        <v>1459</v>
+        <v>1463</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>55.06</v>
+        <v>55.76</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>17.24</v>
+        <v>17.13</v>
       </c>
       <c r="L56" s="3" t="n">
-        <v>9.49</v>
+        <v>10.32</v>
       </c>
       <c r="M56" s="3" t="n">
-        <v>23.92</v>
+        <v>24.63</v>
       </c>
     </row>
     <row r="57">
@@ -2610,38 +2610,38 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>SRR26147396</t>
+          <t>SRR26147395</t>
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>24827</v>
+        <v>23407</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>35493959</v>
+        <v>33487460</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>1429.65</v>
+        <v>1430.66</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>3556</v>
+        <v>4013</v>
       </c>
       <c r="I57" s="3" t="n">
         <v>1459</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>55.2</v>
+        <v>55.06</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>17.2</v>
+        <v>17.24</v>
       </c>
       <c r="L57" s="3" t="n">
-        <v>9.220000000000001</v>
+        <v>9.49</v>
       </c>
       <c r="M57" s="3" t="n">
-        <v>26.17</v>
+        <v>23.92</v>
       </c>
     </row>
     <row r="58">
@@ -2650,38 +2650,38 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>SRR26147397</t>
+          <t>SRR26147396</t>
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>19635</v>
+        <v>24827</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>28271647</v>
+        <v>35493959</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>1439.86</v>
+        <v>1429.65</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>4138</v>
+        <v>3556</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>1460</v>
+        <v>1459</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>54.89</v>
+        <v>55.2</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>17.23</v>
+        <v>17.2</v>
       </c>
       <c r="L58" s="3" t="n">
-        <v>9.35</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="M58" s="3" t="n">
-        <v>24.14</v>
+        <v>26.17</v>
       </c>
     </row>
     <row r="59">
@@ -2690,38 +2690,38 @@
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>SRR26147398</t>
+          <t>SRR26147397</t>
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>21843</v>
+        <v>19635</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>31495884</v>
+        <v>28271647</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>1441.92</v>
+        <v>1439.86</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>2889</v>
+        <v>4138</v>
       </c>
       <c r="I59" s="3" t="n">
-        <v>1458</v>
+        <v>1460</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>54.76</v>
+        <v>54.89</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>17.3</v>
+        <v>17.23</v>
       </c>
       <c r="L59" s="3" t="n">
-        <v>10.15</v>
+        <v>9.35</v>
       </c>
       <c r="M59" s="3" t="n">
-        <v>25.58</v>
+        <v>24.14</v>
       </c>
     </row>
     <row r="60">
@@ -2730,38 +2730,38 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>SRR26147399</t>
+          <t>SRR26147398</t>
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>26323</v>
+        <v>21843</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>37942971</v>
+        <v>31495884</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>1441.44</v>
+        <v>1441.92</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>3986</v>
+        <v>2889</v>
       </c>
       <c r="I60" s="3" t="n">
-        <v>1459</v>
+        <v>1458</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>55.33</v>
+        <v>54.76</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>17.29</v>
+        <v>17.3</v>
       </c>
       <c r="L60" s="3" t="n">
-        <v>10.01</v>
+        <v>10.15</v>
       </c>
       <c r="M60" s="3" t="n">
-        <v>26.18</v>
+        <v>25.58</v>
       </c>
     </row>
     <row r="61">
@@ -2770,38 +2770,38 @@
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>SRR26147400</t>
+          <t>SRR26147399</t>
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>22930</v>
+        <v>26323</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>33101994</v>
+        <v>37942971</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>1443.61</v>
+        <v>1441.44</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>6165</v>
+        <v>3986</v>
       </c>
       <c r="I61" s="3" t="n">
-        <v>1463</v>
+        <v>1459</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>56.09</v>
+        <v>55.33</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>17.17</v>
+        <v>17.29</v>
       </c>
       <c r="L61" s="3" t="n">
-        <v>10.61</v>
+        <v>10.01</v>
       </c>
       <c r="M61" s="3" t="n">
-        <v>25.18</v>
+        <v>26.18</v>
       </c>
     </row>
     <row r="62">
@@ -2810,38 +2810,38 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>SRR26147401</t>
+          <t>SRR26147400</t>
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>20726</v>
+        <v>22930</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>29830327</v>
+        <v>33101994</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>1439.27</v>
+        <v>1443.61</v>
       </c>
       <c r="G62" s="3" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>3078</v>
+        <v>6165</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>1464</v>
+        <v>1463</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>56.07</v>
+        <v>56.09</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>17.24</v>
+        <v>17.17</v>
       </c>
       <c r="L62" s="3" t="n">
-        <v>10.67</v>
+        <v>10.61</v>
       </c>
       <c r="M62" s="3" t="n">
-        <v>25.36</v>
+        <v>25.18</v>
       </c>
     </row>
     <row r="63">
@@ -2850,38 +2850,38 @@
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>SRR26147402</t>
+          <t>SRR26147401</t>
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>22382</v>
+        <v>20726</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>32222846</v>
+        <v>29830327</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>1439.68</v>
+        <v>1439.27</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>3622</v>
+        <v>3078</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>1461</v>
+        <v>1464</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>56.12</v>
+        <v>56.07</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>17.17</v>
+        <v>17.24</v>
       </c>
       <c r="L63" s="3" t="n">
-        <v>10.27</v>
+        <v>10.67</v>
       </c>
       <c r="M63" s="3" t="n">
-        <v>24.35</v>
+        <v>25.36</v>
       </c>
     </row>
     <row r="64">
@@ -2890,38 +2890,38 @@
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>SRR26147403</t>
+          <t>SRR26147402</t>
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>29062</v>
+        <v>22382</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>41948000</v>
+        <v>32222846</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>1443.4</v>
+        <v>1439.68</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>5167</v>
+        <v>3622</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>1462</v>
+        <v>1461</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>55.92</v>
+        <v>56.12</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>17.15</v>
+        <v>17.17</v>
       </c>
       <c r="L64" s="3" t="n">
-        <v>10.52</v>
+        <v>10.27</v>
       </c>
       <c r="M64" s="3" t="n">
-        <v>23.93</v>
+        <v>24.35</v>
       </c>
     </row>
     <row r="65">
@@ -2930,38 +2930,38 @@
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>SRR26147404</t>
+          <t>SRR26147403</t>
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>16696</v>
+        <v>29062</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>24066553</v>
+        <v>41948000</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>1441.46</v>
+        <v>1443.4</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>3601</v>
+        <v>5167</v>
       </c>
       <c r="I65" s="3" t="n">
-        <v>1464</v>
+        <v>1462</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>55.75</v>
+        <v>55.92</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>17.2</v>
+        <v>17.15</v>
       </c>
       <c r="L65" s="3" t="n">
-        <v>9.550000000000001</v>
+        <v>10.52</v>
       </c>
       <c r="M65" s="3" t="n">
-        <v>24.03</v>
+        <v>23.93</v>
       </c>
     </row>
     <row r="66">
@@ -2970,38 +2970,38 @@
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>SRR26147405</t>
+          <t>SRR26147404</t>
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>14093</v>
+        <v>16696</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>20177217</v>
+        <v>24066553</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>1431.72</v>
+        <v>1441.46</v>
       </c>
       <c r="G66" s="3" t="n">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>4011</v>
+        <v>3601</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>1462</v>
+        <v>1464</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>55.71</v>
+        <v>55.75</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>17.29</v>
+        <v>17.2</v>
       </c>
       <c r="L66" s="3" t="n">
-        <v>10.28</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="M66" s="3" t="n">
-        <v>24.01</v>
+        <v>24.03</v>
       </c>
     </row>
     <row r="67">
@@ -3010,38 +3010,38 @@
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>SRR26147406</t>
+          <t>SRR26147405</t>
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>24896</v>
+        <v>14093</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>35856921</v>
+        <v>20177217</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>1440.27</v>
+        <v>1431.72</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>3758</v>
+        <v>4011</v>
       </c>
       <c r="I67" s="3" t="n">
-        <v>1464</v>
+        <v>1462</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>55.78</v>
+        <v>55.71</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>17.18</v>
+        <v>17.29</v>
       </c>
       <c r="L67" s="3" t="n">
-        <v>10.26</v>
+        <v>10.28</v>
       </c>
       <c r="M67" s="3" t="n">
-        <v>24.88</v>
+        <v>24.01</v>
       </c>
     </row>
     <row r="68">
@@ -3050,38 +3050,38 @@
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>SRR26147407</t>
+          <t>SRR26147406</t>
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>25447</v>
+        <v>24896</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>36772755</v>
+        <v>35856921</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>1445.07</v>
+        <v>1440.27</v>
       </c>
       <c r="G68" s="3" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>3089</v>
+        <v>3758</v>
       </c>
       <c r="I68" s="3" t="n">
         <v>1464</v>
       </c>
       <c r="J68" s="3" t="n">
-        <v>55.92</v>
+        <v>55.78</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>17.22</v>
+        <v>17.18</v>
       </c>
       <c r="L68" s="3" t="n">
-        <v>10.66</v>
+        <v>10.26</v>
       </c>
       <c r="M68" s="3" t="n">
-        <v>24.97</v>
+        <v>24.88</v>
       </c>
     </row>
     <row r="69">
@@ -3090,38 +3090,38 @@
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>SRR26147408</t>
+          <t>SRR26147407</t>
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>13930</v>
+        <v>25447</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>20125563</v>
+        <v>36772755</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>1444.76</v>
+        <v>1445.07</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>3134</v>
+        <v>3089</v>
       </c>
       <c r="I69" s="3" t="n">
         <v>1464</v>
       </c>
       <c r="J69" s="3" t="n">
-        <v>55.97</v>
+        <v>55.92</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>17.2</v>
+        <v>17.22</v>
       </c>
       <c r="L69" s="3" t="n">
-        <v>10.33</v>
+        <v>10.66</v>
       </c>
       <c r="M69" s="3" t="n">
-        <v>24.26</v>
+        <v>24.97</v>
       </c>
     </row>
     <row r="70">
@@ -3130,38 +3130,38 @@
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>SRR26147409</t>
+          <t>SRR26147408</t>
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>25366</v>
+        <v>13930</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>36545308</v>
+        <v>20125563</v>
       </c>
       <c r="F70" s="3" t="n">
-        <v>1440.72</v>
+        <v>1444.76</v>
       </c>
       <c r="G70" s="3" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>3376</v>
+        <v>3134</v>
       </c>
       <c r="I70" s="3" t="n">
-        <v>1461</v>
+        <v>1464</v>
       </c>
       <c r="J70" s="3" t="n">
-        <v>55.04</v>
+        <v>55.97</v>
       </c>
       <c r="K70" s="3" t="n">
-        <v>17.33</v>
+        <v>17.2</v>
       </c>
       <c r="L70" s="3" t="n">
-        <v>9.94</v>
+        <v>10.33</v>
       </c>
       <c r="M70" s="3" t="n">
-        <v>26.8</v>
+        <v>24.26</v>
       </c>
     </row>
     <row r="71">
@@ -3170,38 +3170,38 @@
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>SRR26147410</t>
+          <t>SRR26147409</t>
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>34129</v>
+        <v>25366</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>49063911</v>
+        <v>36545308</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>1437.6</v>
+        <v>1440.72</v>
       </c>
       <c r="G71" s="3" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>6185</v>
+        <v>3376</v>
       </c>
       <c r="I71" s="3" t="n">
-        <v>1459</v>
+        <v>1461</v>
       </c>
       <c r="J71" s="3" t="n">
-        <v>54.92</v>
+        <v>55.04</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>17.25</v>
+        <v>17.33</v>
       </c>
       <c r="L71" s="3" t="n">
-        <v>9.130000000000001</v>
+        <v>9.94</v>
       </c>
       <c r="M71" s="3" t="n">
-        <v>23.93</v>
+        <v>26.8</v>
       </c>
     </row>
     <row r="72">
@@ -3210,38 +3210,38 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>SRR26147411</t>
+          <t>SRR26147410</t>
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>36556</v>
+        <v>34129</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>52125944</v>
+        <v>49063911</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>1425.92</v>
+        <v>1437.6</v>
       </c>
       <c r="G72" s="3" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>4002</v>
+        <v>6185</v>
       </c>
       <c r="I72" s="3" t="n">
-        <v>1458</v>
+        <v>1459</v>
       </c>
       <c r="J72" s="3" t="n">
-        <v>54.88</v>
+        <v>54.92</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>17.3</v>
+        <v>17.25</v>
       </c>
       <c r="L72" s="3" t="n">
-        <v>8.359999999999999</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="M72" s="3" t="n">
-        <v>24.59</v>
+        <v>23.93</v>
       </c>
     </row>
     <row r="73">
@@ -3250,38 +3250,38 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>SRR26147412</t>
+          <t>SRR26147411</t>
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>21163</v>
+        <v>36556</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>30321407</v>
+        <v>52125944</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>1432.76</v>
+        <v>1425.92</v>
       </c>
       <c r="G73" s="3" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>4260</v>
+        <v>4002</v>
       </c>
       <c r="I73" s="3" t="n">
-        <v>1459</v>
+        <v>1458</v>
       </c>
       <c r="J73" s="3" t="n">
-        <v>54.86</v>
+        <v>54.88</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>17.29</v>
+        <v>17.3</v>
       </c>
       <c r="L73" s="3" t="n">
-        <v>9.56</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="M73" s="3" t="n">
-        <v>24.74</v>
+        <v>24.59</v>
       </c>
     </row>
     <row r="74">
@@ -3290,38 +3290,38 @@
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>SRR26147413</t>
+          <t>SRR26147412</t>
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>29845</v>
+        <v>21163</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>42705810</v>
+        <v>30321407</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>1430.92</v>
+        <v>1432.76</v>
       </c>
       <c r="G74" s="3" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>4389</v>
+        <v>4260</v>
       </c>
       <c r="I74" s="3" t="n">
         <v>1459</v>
       </c>
       <c r="J74" s="3" t="n">
-        <v>54.9</v>
+        <v>54.86</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>17.23</v>
+        <v>17.29</v>
       </c>
       <c r="L74" s="3" t="n">
-        <v>9.869999999999999</v>
+        <v>9.56</v>
       </c>
       <c r="M74" s="3" t="n">
-        <v>25.24</v>
+        <v>24.74</v>
       </c>
     </row>
     <row r="75">
@@ -3330,38 +3330,38 @@
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>SRR26147414</t>
+          <t>SRR26147413</t>
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>21128</v>
+        <v>29845</v>
       </c>
       <c r="E75" s="3" t="n">
-        <v>30162791</v>
+        <v>42705810</v>
       </c>
       <c r="F75" s="3" t="n">
-        <v>1427.62</v>
+        <v>1430.92</v>
       </c>
       <c r="G75" s="3" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>3358</v>
+        <v>4389</v>
       </c>
       <c r="I75" s="3" t="n">
         <v>1459</v>
       </c>
       <c r="J75" s="3" t="n">
-        <v>54.83</v>
+        <v>54.9</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>17.27</v>
+        <v>17.23</v>
       </c>
       <c r="L75" s="3" t="n">
-        <v>9.4</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="M75" s="3" t="n">
-        <v>25.43</v>
+        <v>25.24</v>
       </c>
     </row>
     <row r="76">
@@ -3370,38 +3370,38 @@
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>SRR26147415</t>
+          <t>SRR26147414</t>
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>18198</v>
+        <v>21128</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>25955509</v>
+        <v>30162791</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>1426.28</v>
+        <v>1427.62</v>
       </c>
       <c r="G76" s="3" t="n">
         <v>71</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>3506</v>
+        <v>3358</v>
       </c>
       <c r="I76" s="3" t="n">
-        <v>1458</v>
+        <v>1459</v>
       </c>
       <c r="J76" s="3" t="n">
-        <v>54.7</v>
+        <v>54.83</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>17.29</v>
+        <v>17.27</v>
       </c>
       <c r="L76" s="3" t="n">
-        <v>9.789999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="M76" s="3" t="n">
-        <v>24.53</v>
+        <v>25.43</v>
       </c>
     </row>
     <row r="77">
@@ -3410,38 +3410,38 @@
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>SRR26147416</t>
+          <t>SRR26147415</t>
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>12622</v>
+        <v>18198</v>
       </c>
       <c r="E77" s="3" t="n">
-        <v>18110352</v>
+        <v>25955509</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>1434.82</v>
+        <v>1426.28</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>4065</v>
+        <v>3506</v>
       </c>
       <c r="I77" s="3" t="n">
-        <v>1463</v>
+        <v>1458</v>
       </c>
       <c r="J77" s="3" t="n">
-        <v>55.86</v>
+        <v>54.7</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>17.17</v>
+        <v>17.29</v>
       </c>
       <c r="L77" s="3" t="n">
-        <v>10.23</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="M77" s="3" t="n">
-        <v>25.74</v>
+        <v>24.53</v>
       </c>
     </row>
     <row r="78">
@@ -3450,38 +3450,38 @@
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>SRR26147417</t>
+          <t>SRR26147416</t>
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>43819</v>
+        <v>12622</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>63159927</v>
+        <v>18110352</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>1441.38</v>
+        <v>1434.82</v>
       </c>
       <c r="G78" s="3" t="n">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>3848</v>
+        <v>4065</v>
       </c>
       <c r="I78" s="3" t="n">
-        <v>1459</v>
+        <v>1463</v>
       </c>
       <c r="J78" s="3" t="n">
-        <v>55.07</v>
+        <v>55.86</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>17.24</v>
+        <v>17.17</v>
       </c>
       <c r="L78" s="3" t="n">
-        <v>10.25</v>
+        <v>10.23</v>
       </c>
       <c r="M78" s="3" t="n">
-        <v>24.67</v>
+        <v>25.74</v>
       </c>
     </row>
     <row r="79">
@@ -3490,38 +3490,38 @@
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>SRR26147418</t>
+          <t>SRR26147417</t>
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>32495</v>
+        <v>43819</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>46773666</v>
+        <v>63159927</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>1439.41</v>
+        <v>1441.38</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>3166</v>
+        <v>3848</v>
       </c>
       <c r="I79" s="3" t="n">
-        <v>1463</v>
+        <v>1459</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>56.18</v>
+        <v>55.07</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>17.18</v>
+        <v>17.24</v>
       </c>
       <c r="L79" s="3" t="n">
-        <v>10.34</v>
+        <v>10.25</v>
       </c>
       <c r="M79" s="3" t="n">
-        <v>24.06</v>
+        <v>24.67</v>
       </c>
     </row>
     <row r="80">
@@ -3530,38 +3530,38 @@
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>SRR26147421</t>
+          <t>SRR26147418</t>
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>36236</v>
+        <v>32495</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>51846332</v>
+        <v>46773666</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>1430.8</v>
+        <v>1439.41</v>
       </c>
       <c r="G80" s="3" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>4318</v>
+        <v>3166</v>
       </c>
       <c r="I80" s="3" t="n">
-        <v>1458</v>
+        <v>1463</v>
       </c>
       <c r="J80" s="3" t="n">
-        <v>54.4</v>
+        <v>56.18</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>17.28</v>
+        <v>17.18</v>
       </c>
       <c r="L80" s="3" t="n">
-        <v>9.359999999999999</v>
+        <v>10.34</v>
       </c>
       <c r="M80" s="3" t="n">
-        <v>27.11</v>
+        <v>24.06</v>
       </c>
     </row>
     <row r="81">
@@ -3570,38 +3570,38 @@
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>SRR26147432</t>
+          <t>SRR26147421</t>
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>30426</v>
+        <v>36236</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>43456912</v>
+        <v>51846332</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>1428.28</v>
+        <v>1430.8</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>3727</v>
+        <v>4318</v>
       </c>
       <c r="I81" s="3" t="n">
-        <v>1459</v>
+        <v>1458</v>
       </c>
       <c r="J81" s="3" t="n">
-        <v>54.57</v>
+        <v>54.4</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>17.25</v>
+        <v>17.28</v>
       </c>
       <c r="L81" s="3" t="n">
-        <v>9.220000000000001</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="M81" s="3" t="n">
-        <v>24.28</v>
+        <v>27.11</v>
       </c>
     </row>
     <row r="82">
@@ -3610,38 +3610,38 @@
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>SRR26147443</t>
+          <t>SRR26147432</t>
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>19751</v>
+        <v>30426</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>28203162</v>
+        <v>43456912</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>1427.94</v>
+        <v>1428.28</v>
       </c>
       <c r="G82" s="3" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>3589</v>
+        <v>3727</v>
       </c>
       <c r="I82" s="3" t="n">
         <v>1459</v>
       </c>
       <c r="J82" s="3" t="n">
-        <v>54.54</v>
+        <v>54.57</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>17.27</v>
+        <v>17.25</v>
       </c>
       <c r="L82" s="3" t="n">
-        <v>9.77</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="M82" s="3" t="n">
-        <v>25.31</v>
+        <v>24.28</v>
       </c>
     </row>
     <row r="83">
@@ -3650,38 +3650,38 @@
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>SRR26147458</t>
+          <t>SRR26147443</t>
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>21634</v>
+        <v>19751</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>31324575</v>
+        <v>28203162</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>1447.93</v>
+        <v>1427.94</v>
       </c>
       <c r="G83" s="3" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>3129</v>
+        <v>3589</v>
       </c>
       <c r="I83" s="3" t="n">
-        <v>1464</v>
+        <v>1459</v>
       </c>
       <c r="J83" s="3" t="n">
-        <v>55.84</v>
+        <v>54.54</v>
       </c>
       <c r="K83" s="3" t="n">
         <v>17.27</v>
       </c>
       <c r="L83" s="3" t="n">
-        <v>10.29</v>
+        <v>9.77</v>
       </c>
       <c r="M83" s="3" t="n">
-        <v>24.25</v>
+        <v>25.31</v>
       </c>
     </row>
     <row r="84">
@@ -3690,38 +3690,38 @@
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>SRR26147469</t>
+          <t>SRR26147458</t>
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>21620</v>
+        <v>21634</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>31199117</v>
+        <v>31324575</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>1443.07</v>
+        <v>1447.93</v>
       </c>
       <c r="G84" s="3" t="n">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>4060</v>
+        <v>3129</v>
       </c>
       <c r="I84" s="3" t="n">
         <v>1464</v>
       </c>
       <c r="J84" s="3" t="n">
-        <v>56.08</v>
+        <v>55.84</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>17.18</v>
+        <v>17.27</v>
       </c>
       <c r="L84" s="3" t="n">
-        <v>8.44</v>
+        <v>10.29</v>
       </c>
       <c r="M84" s="3" t="n">
-        <v>24.52</v>
+        <v>24.25</v>
       </c>
     </row>
     <row r="85">
@@ -3730,38 +3730,38 @@
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>SRR26147470</t>
+          <t>SRR26147469</t>
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>15172</v>
+        <v>21620</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>22387697</v>
+        <v>31199117</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>1475.59</v>
+        <v>1443.07</v>
       </c>
       <c r="G85" s="3" t="n">
-        <v>272</v>
+        <v>78</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>3936</v>
+        <v>4060</v>
       </c>
       <c r="I85" s="3" t="n">
-        <v>1477</v>
+        <v>1464</v>
       </c>
       <c r="J85" s="3" t="n">
-        <v>54.33</v>
+        <v>56.08</v>
       </c>
       <c r="K85" s="3" t="n">
         <v>17.18</v>
       </c>
       <c r="L85" s="3" t="n">
-        <v>10.59</v>
+        <v>8.44</v>
       </c>
       <c r="M85" s="3" t="n">
-        <v>23.43</v>
+        <v>24.52</v>
       </c>
     </row>
     <row r="86">
@@ -3770,38 +3770,38 @@
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>SRR26147481</t>
+          <t>SRR26147470</t>
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>20487</v>
+        <v>15172</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>29644201</v>
+        <v>22387697</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>1446.98</v>
+        <v>1475.59</v>
       </c>
       <c r="G86" s="3" t="n">
-        <v>78</v>
+        <v>272</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>4108</v>
+        <v>3936</v>
       </c>
       <c r="I86" s="3" t="n">
-        <v>1465</v>
+        <v>1477</v>
       </c>
       <c r="J86" s="3" t="n">
-        <v>56.19</v>
+        <v>54.33</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>17.2</v>
+        <v>17.18</v>
       </c>
       <c r="L86" s="3" t="n">
-        <v>10.53</v>
+        <v>10.59</v>
       </c>
       <c r="M86" s="3" t="n">
-        <v>23.4</v>
+        <v>23.43</v>
       </c>
     </row>
     <row r="87">
@@ -3810,38 +3810,38 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>SRR26147483</t>
+          <t>SRR26147481</t>
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>25120</v>
+        <v>20487</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>35697825</v>
+        <v>29644201</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>1421.09</v>
+        <v>1446.98</v>
       </c>
       <c r="G87" s="3" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H87" s="3" t="n">
-        <v>4239</v>
+        <v>4108</v>
       </c>
       <c r="I87" s="3" t="n">
-        <v>1458</v>
+        <v>1465</v>
       </c>
       <c r="J87" s="3" t="n">
-        <v>53.84</v>
+        <v>56.19</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>17.32</v>
+        <v>17.2</v>
       </c>
       <c r="L87" s="3" t="n">
-        <v>10.36</v>
+        <v>10.53</v>
       </c>
       <c r="M87" s="3" t="n">
-        <v>24.24</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="88">
@@ -3850,38 +3850,38 @@
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>SRR26147494</t>
+          <t>SRR26147483</t>
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>30646</v>
+        <v>25120</v>
       </c>
       <c r="E88" s="3" t="n">
-        <v>43900163</v>
+        <v>35697825</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>1432.49</v>
+        <v>1421.09</v>
       </c>
       <c r="G88" s="3" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H88" s="3" t="n">
-        <v>3366</v>
+        <v>4239</v>
       </c>
       <c r="I88" s="3" t="n">
         <v>1458</v>
       </c>
       <c r="J88" s="3" t="n">
-        <v>53.8</v>
+        <v>53.84</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>17.33</v>
+        <v>17.32</v>
       </c>
       <c r="L88" s="3" t="n">
-        <v>10.41</v>
+        <v>10.36</v>
       </c>
       <c r="M88" s="3" t="n">
-        <v>25.19</v>
+        <v>24.24</v>
       </c>
     </row>
     <row r="89">
@@ -3890,38 +3890,38 @@
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>SRR26147505</t>
+          <t>SRR26147494</t>
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>27985</v>
+        <v>30646</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>40257718</v>
+        <v>43900163</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>1438.55</v>
+        <v>1432.49</v>
       </c>
       <c r="G89" s="3" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>3478</v>
+        <v>3366</v>
       </c>
       <c r="I89" s="3" t="n">
-        <v>1459</v>
+        <v>1458</v>
       </c>
       <c r="J89" s="3" t="n">
-        <v>53.96</v>
+        <v>53.8</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>17.38</v>
+        <v>17.33</v>
       </c>
       <c r="L89" s="3" t="n">
-        <v>9</v>
+        <v>10.41</v>
       </c>
       <c r="M89" s="3" t="n">
-        <v>24.3</v>
+        <v>25.19</v>
       </c>
     </row>
     <row r="90">
@@ -3930,334 +3930,374 @@
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
+          <t>SRR26147505</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>27985</v>
+      </c>
+      <c r="E90" s="3" t="n">
+        <v>40257718</v>
+      </c>
+      <c r="F90" s="3" t="n">
+        <v>1438.55</v>
+      </c>
+      <c r="G90" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="H90" s="3" t="n">
+        <v>3478</v>
+      </c>
+      <c r="I90" s="3" t="n">
+        <v>1459</v>
+      </c>
+      <c r="J90" s="3" t="n">
+        <v>53.96</v>
+      </c>
+      <c r="K90" s="3" t="n">
+        <v>17.38</v>
+      </c>
+      <c r="L90" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="M90" s="3" t="n">
+        <v>24.3</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="11" t="n">
+        <v>89</v>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
           <t>SRR26147516</t>
         </is>
       </c>
-      <c r="D90" s="3" t="n">
+      <c r="D91" s="3" t="n">
         <v>40466</v>
       </c>
-      <c r="E90" s="3" t="n">
+      <c r="E91" s="3" t="n">
         <v>58130904</v>
       </c>
-      <c r="F90" s="3" t="n">
+      <c r="F91" s="3" t="n">
         <v>1436.54</v>
       </c>
-      <c r="G90" s="3" t="n">
+      <c r="G91" s="3" t="n">
         <v>73</v>
       </c>
-      <c r="H90" s="3" t="n">
+      <c r="H91" s="3" t="n">
         <v>4352</v>
       </c>
-      <c r="I90" s="3" t="n">
+      <c r="I91" s="3" t="n">
         <v>1463</v>
       </c>
-      <c r="J90" s="3" t="n">
+      <c r="J91" s="3" t="n">
         <v>56.12</v>
       </c>
-      <c r="K90" s="3" t="n">
+      <c r="K91" s="3" t="n">
         <v>17.1</v>
       </c>
-      <c r="L90" s="3" t="n">
+      <c r="L91" s="3" t="n">
         <v>9.550000000000001</v>
       </c>
-      <c r="M90" s="3" t="n">
+      <c r="M91" s="3" t="n">
         <v>24.52</v>
       </c>
     </row>
-    <row r="91">
-      <c r="C91" s="11" t="inlineStr">
+    <row r="92">
+      <c r="C92" s="11" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D91" s="10">
-        <f>SUM(D3:D90)</f>
+      <c r="D92" s="10">
+        <f>SUM(D3:D91)</f>
         <v/>
       </c>
-      <c r="E91" s="10">
-        <f>SUM(E3:E90)</f>
+      <c r="E92" s="10">
+        <f>SUM(E3:E91)</f>
         <v/>
       </c>
-      <c r="F91" s="10" t="inlineStr">
+      <c r="F92" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G91" s="10" t="inlineStr">
+      <c r="G92" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H91" s="10" t="inlineStr">
+      <c r="H92" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I91" s="10" t="inlineStr">
+      <c r="I92" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J91" s="10" t="inlineStr">
+      <c r="J92" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K91" s="10" t="inlineStr">
+      <c r="K92" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="L91" s="10" t="inlineStr">
+      <c r="L92" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M91" s="10" t="inlineStr">
+      <c r="M92" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="C92" s="12" t="n"/>
-      <c r="D92" s="12" t="n"/>
-      <c r="E92" s="12" t="n"/>
-      <c r="F92" s="12" t="n"/>
-      <c r="G92" s="12" t="n"/>
-      <c r="H92" s="12" t="n"/>
-      <c r="I92" s="12" t="n"/>
-      <c r="J92" s="12" t="n"/>
-      <c r="K92" s="12" t="n"/>
-      <c r="L92" s="12" t="n"/>
-      <c r="M92" s="12" t="n"/>
-    </row>
     <row r="93">
-      <c r="C93" s="11" t="inlineStr">
+      <c r="C93" s="12" t="n"/>
+      <c r="D93" s="12" t="n"/>
+      <c r="E93" s="12" t="n"/>
+      <c r="F93" s="12" t="n"/>
+      <c r="G93" s="12" t="n"/>
+      <c r="H93" s="12" t="n"/>
+      <c r="I93" s="12" t="n"/>
+      <c r="J93" s="12" t="n"/>
+      <c r="K93" s="12" t="n"/>
+      <c r="L93" s="12" t="n"/>
+      <c r="M93" s="12" t="n"/>
+    </row>
+    <row r="94">
+      <c r="C94" s="11" t="inlineStr">
         <is>
           <t>PROMEDIO</t>
         </is>
       </c>
-      <c r="D93" s="10">
-        <f>AVERAGE(D3:D90)</f>
+      <c r="D94" s="10">
+        <f>AVERAGE(D3:D91)</f>
         <v/>
       </c>
-      <c r="E93" s="10">
-        <f>AVERAGE(E3:E90)</f>
+      <c r="E94" s="10">
+        <f>AVERAGE(E3:E91)</f>
         <v/>
       </c>
-      <c r="F93" s="10">
-        <f>AVERAGE(F3:F90)</f>
+      <c r="F94" s="10">
+        <f>AVERAGE(F3:F91)</f>
         <v/>
       </c>
-      <c r="G93" s="10">
-        <f>AVERAGE(G3:G90)</f>
+      <c r="G94" s="10">
+        <f>AVERAGE(G3:G91)</f>
         <v/>
       </c>
-      <c r="H93" s="10">
-        <f>AVERAGE(H3:H90)</f>
+      <c r="H94" s="10">
+        <f>AVERAGE(H3:H91)</f>
         <v/>
       </c>
-      <c r="I93" s="10">
-        <f>AVERAGE(I3:I90)</f>
+      <c r="I94" s="10">
+        <f>AVERAGE(I3:I91)</f>
         <v/>
       </c>
-      <c r="J93" s="10">
-        <f>AVERAGE(J3:J90)</f>
+      <c r="J94" s="10">
+        <f>AVERAGE(J3:J91)</f>
         <v/>
       </c>
-      <c r="K93" s="10">
-        <f>AVERAGE(K3:K90)</f>
+      <c r="K94" s="10">
+        <f>AVERAGE(K3:K91)</f>
         <v/>
       </c>
-      <c r="L93" s="10">
-        <f>AVERAGE(L3:L90)</f>
+      <c r="L94" s="10">
+        <f>AVERAGE(L3:L91)</f>
         <v/>
       </c>
-      <c r="M93" s="10">
-        <f>AVERAGE(M3:M90)</f>
+      <c r="M94" s="10">
+        <f>AVERAGE(M3:M91)</f>
         <v/>
       </c>
     </row>
-    <row r="94">
-      <c r="C94" s="12" t="n"/>
-      <c r="D94" s="12" t="n"/>
-      <c r="E94" s="12" t="n"/>
-      <c r="F94" s="12" t="n"/>
-      <c r="G94" s="12" t="n"/>
-      <c r="H94" s="12" t="n"/>
-      <c r="I94" s="12" t="n"/>
-      <c r="J94" s="12" t="n"/>
-      <c r="K94" s="12" t="n"/>
-      <c r="L94" s="12" t="n"/>
-      <c r="M94" s="12" t="n"/>
-    </row>
     <row r="95">
-      <c r="C95" s="11" t="inlineStr">
+      <c r="C95" s="12" t="n"/>
+      <c r="D95" s="12" t="n"/>
+      <c r="E95" s="12" t="n"/>
+      <c r="F95" s="12" t="n"/>
+      <c r="G95" s="12" t="n"/>
+      <c r="H95" s="12" t="n"/>
+      <c r="I95" s="12" t="n"/>
+      <c r="J95" s="12" t="n"/>
+      <c r="K95" s="12" t="n"/>
+      <c r="L95" s="12" t="n"/>
+      <c r="M95" s="12" t="n"/>
+    </row>
+    <row r="96">
+      <c r="C96" s="11" t="inlineStr">
         <is>
           <t>MÁXIMO</t>
         </is>
       </c>
-      <c r="D95" s="10">
-        <f>MAX(D3:D90)</f>
+      <c r="D96" s="10">
+        <f>MAX(D3:D91)</f>
         <v/>
       </c>
-      <c r="E95" s="10">
-        <f>MAX(E3:E90)</f>
+      <c r="E96" s="10">
+        <f>MAX(E3:E91)</f>
         <v/>
       </c>
-      <c r="F95" s="10">
-        <f>MAX(F3:F90)</f>
+      <c r="F96" s="10">
+        <f>MAX(F3:F91)</f>
         <v/>
       </c>
-      <c r="G95" s="10">
-        <f>MAX(G3:G90)</f>
+      <c r="G96" s="10">
+        <f>MAX(G3:G91)</f>
         <v/>
       </c>
-      <c r="H95" s="10">
-        <f>MAX(H3:H90)</f>
+      <c r="H96" s="10">
+        <f>MAX(H3:H91)</f>
         <v/>
       </c>
-      <c r="I95" s="10">
-        <f>MAX(I3:I90)</f>
+      <c r="I96" s="10">
+        <f>MAX(I3:I91)</f>
         <v/>
       </c>
-      <c r="J95" s="10">
-        <f>MAX(J3:J90)</f>
+      <c r="J96" s="10">
+        <f>MAX(J3:J91)</f>
         <v/>
       </c>
-      <c r="K95" s="10">
-        <f>MAX(K3:K90)</f>
+      <c r="K96" s="10">
+        <f>MAX(K3:K91)</f>
         <v/>
       </c>
-      <c r="L95" s="10">
-        <f>MAX(L3:L90)</f>
+      <c r="L96" s="10">
+        <f>MAX(L3:L91)</f>
         <v/>
       </c>
-      <c r="M95" s="10">
-        <f>MAX(M3:M90)</f>
+      <c r="M96" s="10">
+        <f>MAX(M3:M91)</f>
         <v/>
       </c>
     </row>
-    <row r="96">
-      <c r="C96" s="12" t="n"/>
-      <c r="D96" s="12" t="n"/>
-      <c r="E96" s="12" t="n"/>
-      <c r="F96" s="12" t="n"/>
-      <c r="G96" s="12" t="n"/>
-      <c r="H96" s="12" t="n"/>
-      <c r="I96" s="12" t="n"/>
-      <c r="J96" s="12" t="n"/>
-      <c r="K96" s="12" t="n"/>
-      <c r="L96" s="12" t="n"/>
-      <c r="M96" s="12" t="n"/>
-    </row>
     <row r="97">
-      <c r="C97" s="11" t="inlineStr">
+      <c r="C97" s="12" t="n"/>
+      <c r="D97" s="12" t="n"/>
+      <c r="E97" s="12" t="n"/>
+      <c r="F97" s="12" t="n"/>
+      <c r="G97" s="12" t="n"/>
+      <c r="H97" s="12" t="n"/>
+      <c r="I97" s="12" t="n"/>
+      <c r="J97" s="12" t="n"/>
+      <c r="K97" s="12" t="n"/>
+      <c r="L97" s="12" t="n"/>
+      <c r="M97" s="12" t="n"/>
+    </row>
+    <row r="98">
+      <c r="C98" s="11" t="inlineStr">
         <is>
           <t>MÍNIMO</t>
         </is>
       </c>
-      <c r="D97" s="10">
-        <f>MIN(D3:D90)</f>
+      <c r="D98" s="10">
+        <f>MIN(D3:D91)</f>
         <v/>
       </c>
-      <c r="E97" s="10">
-        <f>MIN(E3:E90)</f>
+      <c r="E98" s="10">
+        <f>MIN(E3:E91)</f>
         <v/>
       </c>
-      <c r="F97" s="10">
-        <f>MIN(F3:F90)</f>
+      <c r="F98" s="10">
+        <f>MIN(F3:F91)</f>
         <v/>
       </c>
-      <c r="G97" s="10">
-        <f>MIN(G3:G90)</f>
+      <c r="G98" s="10">
+        <f>MIN(G3:G91)</f>
         <v/>
       </c>
-      <c r="H97" s="10">
-        <f>MIN(H3:H90)</f>
+      <c r="H98" s="10">
+        <f>MIN(H3:H91)</f>
         <v/>
       </c>
-      <c r="I97" s="10">
-        <f>MIN(I3:I90)</f>
+      <c r="I98" s="10">
+        <f>MIN(I3:I91)</f>
         <v/>
       </c>
-      <c r="J97" s="10">
-        <f>MIN(J3:J90)</f>
+      <c r="J98" s="10">
+        <f>MIN(J3:J91)</f>
         <v/>
       </c>
-      <c r="K97" s="10">
-        <f>MIN(K3:K90)</f>
+      <c r="K98" s="10">
+        <f>MIN(K3:K91)</f>
         <v/>
       </c>
-      <c r="L97" s="10">
-        <f>MIN(L3:L90)</f>
+      <c r="L98" s="10">
+        <f>MIN(L3:L91)</f>
         <v/>
       </c>
-      <c r="M97" s="10">
-        <f>MIN(M3:M90)</f>
+      <c r="M98" s="10">
+        <f>MIN(M3:M91)</f>
         <v/>
       </c>
     </row>
-    <row r="98">
-      <c r="C98" s="12" t="n"/>
-      <c r="D98" s="12" t="n"/>
-      <c r="E98" s="12" t="n"/>
-      <c r="F98" s="12" t="n"/>
-      <c r="G98" s="12" t="n"/>
-      <c r="H98" s="12" t="n"/>
-      <c r="I98" s="12" t="n"/>
-      <c r="J98" s="12" t="n"/>
-      <c r="K98" s="12" t="n"/>
-      <c r="L98" s="12" t="n"/>
-      <c r="M98" s="12" t="n"/>
+    <row r="99">
+      <c r="C99" s="12" t="n"/>
+      <c r="D99" s="12" t="n"/>
+      <c r="E99" s="12" t="n"/>
+      <c r="F99" s="12" t="n"/>
+      <c r="G99" s="12" t="n"/>
+      <c r="H99" s="12" t="n"/>
+      <c r="I99" s="12" t="n"/>
+      <c r="J99" s="12" t="n"/>
+      <c r="K99" s="12" t="n"/>
+      <c r="L99" s="12" t="n"/>
+      <c r="M99" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="J93:J94"/>
-    <mergeCell ref="L91:L92"/>
-    <mergeCell ref="I95:I96"/>
-    <mergeCell ref="I91:I92"/>
-    <mergeCell ref="K91:K92"/>
-    <mergeCell ref="L97:L98"/>
-    <mergeCell ref="C97:C98"/>
-    <mergeCell ref="H93:H94"/>
-    <mergeCell ref="F95:F96"/>
-    <mergeCell ref="G97:G98"/>
-    <mergeCell ref="L93:L94"/>
-    <mergeCell ref="I97:I98"/>
-    <mergeCell ref="D95:D96"/>
-    <mergeCell ref="F91:F92"/>
-    <mergeCell ref="J95:J96"/>
-    <mergeCell ref="D91:D92"/>
-    <mergeCell ref="J91:J92"/>
-    <mergeCell ref="C93:C94"/>
-    <mergeCell ref="G93:G94"/>
-    <mergeCell ref="I93:I94"/>
-    <mergeCell ref="G95:G96"/>
-    <mergeCell ref="D97:D98"/>
-    <mergeCell ref="F97:F98"/>
-    <mergeCell ref="F93:F94"/>
-    <mergeCell ref="C95:C96"/>
-    <mergeCell ref="E95:E96"/>
-    <mergeCell ref="M95:M96"/>
-    <mergeCell ref="M91:M92"/>
-    <mergeCell ref="C91:C92"/>
-    <mergeCell ref="E91:E92"/>
-    <mergeCell ref="D93:D94"/>
-    <mergeCell ref="G91:G92"/>
-    <mergeCell ref="E97:E98"/>
-    <mergeCell ref="K97:K98"/>
-    <mergeCell ref="M97:M98"/>
-    <mergeCell ref="M93:M94"/>
-    <mergeCell ref="H95:H96"/>
-    <mergeCell ref="H91:H92"/>
-    <mergeCell ref="L95:L96"/>
-    <mergeCell ref="J97:J98"/>
-    <mergeCell ref="E93:E94"/>
-    <mergeCell ref="K93:K94"/>
-    <mergeCell ref="H97:H98"/>
-    <mergeCell ref="K95:K96"/>
+    <mergeCell ref="E92:E93"/>
+    <mergeCell ref="K92:K93"/>
+    <mergeCell ref="D96:D97"/>
+    <mergeCell ref="E98:E99"/>
+    <mergeCell ref="G98:G99"/>
+    <mergeCell ref="C94:C95"/>
+    <mergeCell ref="M98:M99"/>
+    <mergeCell ref="K94:K95"/>
+    <mergeCell ref="M94:M95"/>
+    <mergeCell ref="J98:J99"/>
+    <mergeCell ref="L92:L93"/>
+    <mergeCell ref="E94:E95"/>
+    <mergeCell ref="K96:K97"/>
+    <mergeCell ref="H98:H99"/>
+    <mergeCell ref="F94:F95"/>
+    <mergeCell ref="I92:I93"/>
+    <mergeCell ref="H94:H95"/>
+    <mergeCell ref="I96:I97"/>
+    <mergeCell ref="G92:G93"/>
+    <mergeCell ref="K98:K99"/>
+    <mergeCell ref="J94:J95"/>
+    <mergeCell ref="F96:F97"/>
+    <mergeCell ref="L94:L95"/>
+    <mergeCell ref="D92:D93"/>
+    <mergeCell ref="H96:H97"/>
+    <mergeCell ref="I98:I99"/>
+    <mergeCell ref="F92:F93"/>
+    <mergeCell ref="L96:L97"/>
+    <mergeCell ref="G94:G95"/>
+    <mergeCell ref="C96:C97"/>
+    <mergeCell ref="I94:I95"/>
+    <mergeCell ref="J96:J97"/>
+    <mergeCell ref="H92:H93"/>
+    <mergeCell ref="L98:L99"/>
+    <mergeCell ref="D98:D99"/>
+    <mergeCell ref="G96:G97"/>
+    <mergeCell ref="M96:M97"/>
+    <mergeCell ref="F98:F99"/>
+    <mergeCell ref="D94:D95"/>
+    <mergeCell ref="M92:M93"/>
+    <mergeCell ref="J92:J93"/>
+    <mergeCell ref="E96:E97"/>
+    <mergeCell ref="C98:C99"/>
+    <mergeCell ref="C92:C93"/>
   </mergeCells>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup orientation="portrait" paperSize="9" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Leave the control sample S0A1 (SRR26147470) out of annexes 3, 4 and 7-10
S0A1 is the autoclaved-soil control, so it is no longer processed. It was
also removed from the article side of the taxa comparison (its barcode01).
Pearson is now 0.9924 (family, 125 shared), 0.9886 (genus, 329) and
0.9635 (species, 789). The CS vs CSSwP tests do not change because they
already excluded the control; the PCoA, the distance matrices and the EMU
tables now have 88 samples. Annex 11 never included the control.
</commit_message>
<xml_diff>
--- a/Anexo_03_Estadisticas_pre_limpieza/Anexo_03_Estadisticas_pre_limpieza.xlsx
+++ b/Anexo_03_Estadisticas_pre_limpieza/Anexo_03_Estadisticas_pre_limpieza.xlsx
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:M99"/>
+  <dimension ref="A2:M100"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="13.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col width="13.5703125" customWidth="1" style="1" min="1" max="1"/>
@@ -3770,38 +3770,38 @@
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>SRR26147470</t>
+          <t>SRR26147481</t>
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>15172</v>
+        <v>20487</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>22387697</v>
+        <v>29644201</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>1475.59</v>
+        <v>1446.98</v>
       </c>
       <c r="G86" s="3" t="n">
-        <v>272</v>
+        <v>78</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>3936</v>
+        <v>4108</v>
       </c>
       <c r="I86" s="3" t="n">
-        <v>1477</v>
+        <v>1465</v>
       </c>
       <c r="J86" s="3" t="n">
-        <v>54.33</v>
+        <v>56.19</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>17.18</v>
+        <v>17.2</v>
       </c>
       <c r="L86" s="3" t="n">
-        <v>10.59</v>
+        <v>10.53</v>
       </c>
       <c r="M86" s="3" t="n">
-        <v>23.43</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="87">
@@ -3810,38 +3810,38 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>SRR26147481</t>
+          <t>SRR26147483</t>
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>20487</v>
+        <v>25120</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>29644201</v>
+        <v>35697825</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>1446.98</v>
+        <v>1421.09</v>
       </c>
       <c r="G87" s="3" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H87" s="3" t="n">
-        <v>4108</v>
+        <v>4239</v>
       </c>
       <c r="I87" s="3" t="n">
-        <v>1465</v>
+        <v>1458</v>
       </c>
       <c r="J87" s="3" t="n">
-        <v>56.19</v>
+        <v>53.84</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>17.2</v>
+        <v>17.32</v>
       </c>
       <c r="L87" s="3" t="n">
-        <v>10.53</v>
+        <v>10.36</v>
       </c>
       <c r="M87" s="3" t="n">
-        <v>23.4</v>
+        <v>24.24</v>
       </c>
     </row>
     <row r="88">
@@ -3850,38 +3850,38 @@
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>SRR26147483</t>
+          <t>SRR26147494</t>
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>25120</v>
+        <v>30646</v>
       </c>
       <c r="E88" s="3" t="n">
-        <v>35697825</v>
+        <v>43900163</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>1421.09</v>
+        <v>1432.49</v>
       </c>
       <c r="G88" s="3" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H88" s="3" t="n">
-        <v>4239</v>
+        <v>3366</v>
       </c>
       <c r="I88" s="3" t="n">
         <v>1458</v>
       </c>
       <c r="J88" s="3" t="n">
-        <v>53.84</v>
+        <v>53.8</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>17.32</v>
+        <v>17.33</v>
       </c>
       <c r="L88" s="3" t="n">
-        <v>10.36</v>
+        <v>10.41</v>
       </c>
       <c r="M88" s="3" t="n">
-        <v>24.24</v>
+        <v>25.19</v>
       </c>
     </row>
     <row r="89">
@@ -3890,38 +3890,38 @@
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>SRR26147494</t>
+          <t>SRR26147505</t>
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>30646</v>
+        <v>27985</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>43900163</v>
+        <v>40257718</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>1432.49</v>
+        <v>1438.55</v>
       </c>
       <c r="G89" s="3" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>3366</v>
+        <v>3478</v>
       </c>
       <c r="I89" s="3" t="n">
-        <v>1458</v>
+        <v>1459</v>
       </c>
       <c r="J89" s="3" t="n">
-        <v>53.8</v>
+        <v>53.96</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>17.33</v>
+        <v>17.38</v>
       </c>
       <c r="L89" s="3" t="n">
-        <v>10.41</v>
+        <v>9</v>
       </c>
       <c r="M89" s="3" t="n">
-        <v>25.19</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="90">
@@ -3930,374 +3930,336 @@
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>SRR26147505</t>
+          <t>SRR26147516</t>
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>27985</v>
+        <v>40466</v>
       </c>
       <c r="E90" s="3" t="n">
-        <v>40257718</v>
+        <v>58130904</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>1438.55</v>
+        <v>1436.54</v>
       </c>
       <c r="G90" s="3" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H90" s="3" t="n">
-        <v>3478</v>
+        <v>4352</v>
       </c>
       <c r="I90" s="3" t="n">
-        <v>1459</v>
+        <v>1463</v>
       </c>
       <c r="J90" s="3" t="n">
-        <v>53.96</v>
+        <v>56.12</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>17.38</v>
+        <v>17.1</v>
       </c>
       <c r="L90" s="3" t="n">
-        <v>9</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="M90" s="3" t="n">
-        <v>24.3</v>
+        <v>24.52</v>
       </c>
     </row>
     <row r="91">
-      <c r="B91" s="11" t="n">
-        <v>89</v>
-      </c>
-      <c r="C91" s="7" t="inlineStr">
-        <is>
-          <t>SRR26147516</t>
-        </is>
-      </c>
-      <c r="D91" s="3" t="n">
-        <v>40466</v>
-      </c>
-      <c r="E91" s="3" t="n">
-        <v>58130904</v>
-      </c>
-      <c r="F91" s="3" t="n">
-        <v>1436.54</v>
-      </c>
-      <c r="G91" s="3" t="n">
-        <v>73</v>
-      </c>
-      <c r="H91" s="3" t="n">
-        <v>4352</v>
-      </c>
-      <c r="I91" s="3" t="n">
-        <v>1463</v>
-      </c>
-      <c r="J91" s="3" t="n">
-        <v>56.12</v>
-      </c>
-      <c r="K91" s="3" t="n">
-        <v>17.1</v>
-      </c>
-      <c r="L91" s="3" t="n">
-        <v>9.550000000000001</v>
-      </c>
-      <c r="M91" s="3" t="n">
-        <v>24.52</v>
+      <c r="C91" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D91" s="10">
+        <f>SUM(D3:D90)</f>
+        <v/>
+      </c>
+      <c r="E91" s="10">
+        <f>SUM(E3:E90)</f>
+        <v/>
+      </c>
+      <c r="F91" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G91" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H91" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I91" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J91" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K91" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L91" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M91" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="92">
-      <c r="C92" s="11" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="D92" s="10">
-        <f>SUM(D3:D91)</f>
+      <c r="C92" s="12" t="n"/>
+      <c r="D92" s="12" t="n"/>
+      <c r="E92" s="12" t="n"/>
+      <c r="F92" s="12" t="n"/>
+      <c r="G92" s="12" t="n"/>
+      <c r="H92" s="12" t="n"/>
+      <c r="I92" s="12" t="n"/>
+      <c r="J92" s="12" t="n"/>
+      <c r="K92" s="12" t="n"/>
+      <c r="L92" s="12" t="n"/>
+      <c r="M92" s="12" t="n"/>
+    </row>
+    <row r="93">
+      <c r="C93" s="11" t="inlineStr">
+        <is>
+          <t>PROMEDIO</t>
+        </is>
+      </c>
+      <c r="D93" s="10">
+        <f>AVERAGE(D3:D90)</f>
         <v/>
       </c>
-      <c r="E92" s="10">
-        <f>SUM(E3:E91)</f>
+      <c r="E93" s="10">
+        <f>AVERAGE(E3:E90)</f>
         <v/>
       </c>
-      <c r="F92" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G92" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H92" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I92" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J92" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K92" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L92" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M92" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="C93" s="12" t="n"/>
-      <c r="D93" s="12" t="n"/>
-      <c r="E93" s="12" t="n"/>
-      <c r="F93" s="12" t="n"/>
-      <c r="G93" s="12" t="n"/>
-      <c r="H93" s="12" t="n"/>
-      <c r="I93" s="12" t="n"/>
-      <c r="J93" s="12" t="n"/>
-      <c r="K93" s="12" t="n"/>
-      <c r="L93" s="12" t="n"/>
-      <c r="M93" s="12" t="n"/>
+      <c r="F93" s="10">
+        <f>AVERAGE(F3:F90)</f>
+        <v/>
+      </c>
+      <c r="G93" s="10">
+        <f>AVERAGE(G3:G90)</f>
+        <v/>
+      </c>
+      <c r="H93" s="10">
+        <f>AVERAGE(H3:H90)</f>
+        <v/>
+      </c>
+      <c r="I93" s="10">
+        <f>AVERAGE(I3:I90)</f>
+        <v/>
+      </c>
+      <c r="J93" s="10">
+        <f>AVERAGE(J3:J90)</f>
+        <v/>
+      </c>
+      <c r="K93" s="10">
+        <f>AVERAGE(K3:K90)</f>
+        <v/>
+      </c>
+      <c r="L93" s="10">
+        <f>AVERAGE(L3:L90)</f>
+        <v/>
+      </c>
+      <c r="M93" s="10">
+        <f>AVERAGE(M3:M90)</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
-      <c r="C94" s="11" t="inlineStr">
-        <is>
-          <t>PROMEDIO</t>
-        </is>
-      </c>
-      <c r="D94" s="10">
-        <f>AVERAGE(D3:D91)</f>
+      <c r="C94" s="12" t="n"/>
+      <c r="D94" s="12" t="n"/>
+      <c r="E94" s="12" t="n"/>
+      <c r="F94" s="12" t="n"/>
+      <c r="G94" s="12" t="n"/>
+      <c r="H94" s="12" t="n"/>
+      <c r="I94" s="12" t="n"/>
+      <c r="J94" s="12" t="n"/>
+      <c r="K94" s="12" t="n"/>
+      <c r="L94" s="12" t="n"/>
+      <c r="M94" s="12" t="n"/>
+    </row>
+    <row r="95">
+      <c r="C95" s="11" t="inlineStr">
+        <is>
+          <t>MÁXIMO</t>
+        </is>
+      </c>
+      <c r="D95" s="10">
+        <f>MAX(D3:D90)</f>
         <v/>
       </c>
-      <c r="E94" s="10">
-        <f>AVERAGE(E3:E91)</f>
+      <c r="E95" s="10">
+        <f>MAX(E3:E90)</f>
         <v/>
       </c>
-      <c r="F94" s="10">
-        <f>AVERAGE(F3:F91)</f>
+      <c r="F95" s="10">
+        <f>MAX(F3:F90)</f>
         <v/>
       </c>
-      <c r="G94" s="10">
-        <f>AVERAGE(G3:G91)</f>
+      <c r="G95" s="10">
+        <f>MAX(G3:G90)</f>
         <v/>
       </c>
-      <c r="H94" s="10">
-        <f>AVERAGE(H3:H91)</f>
+      <c r="H95" s="10">
+        <f>MAX(H3:H90)</f>
         <v/>
       </c>
-      <c r="I94" s="10">
-        <f>AVERAGE(I3:I91)</f>
+      <c r="I95" s="10">
+        <f>MAX(I3:I90)</f>
         <v/>
       </c>
-      <c r="J94" s="10">
-        <f>AVERAGE(J3:J91)</f>
+      <c r="J95" s="10">
+        <f>MAX(J3:J90)</f>
         <v/>
       </c>
-      <c r="K94" s="10">
-        <f>AVERAGE(K3:K91)</f>
+      <c r="K95" s="10">
+        <f>MAX(K3:K90)</f>
         <v/>
       </c>
-      <c r="L94" s="10">
-        <f>AVERAGE(L3:L91)</f>
+      <c r="L95" s="10">
+        <f>MAX(L3:L90)</f>
         <v/>
       </c>
-      <c r="M94" s="10">
-        <f>AVERAGE(M3:M91)</f>
+      <c r="M95" s="10">
+        <f>MAX(M3:M90)</f>
         <v/>
       </c>
     </row>
-    <row r="95">
-      <c r="C95" s="12" t="n"/>
-      <c r="D95" s="12" t="n"/>
-      <c r="E95" s="12" t="n"/>
-      <c r="F95" s="12" t="n"/>
-      <c r="G95" s="12" t="n"/>
-      <c r="H95" s="12" t="n"/>
-      <c r="I95" s="12" t="n"/>
-      <c r="J95" s="12" t="n"/>
-      <c r="K95" s="12" t="n"/>
-      <c r="L95" s="12" t="n"/>
-      <c r="M95" s="12" t="n"/>
-    </row>
     <row r="96">
-      <c r="C96" s="11" t="inlineStr">
-        <is>
-          <t>MÁXIMO</t>
-        </is>
-      </c>
-      <c r="D96" s="10">
-        <f>MAX(D3:D91)</f>
+      <c r="C96" s="12" t="n"/>
+      <c r="D96" s="12" t="n"/>
+      <c r="E96" s="12" t="n"/>
+      <c r="F96" s="12" t="n"/>
+      <c r="G96" s="12" t="n"/>
+      <c r="H96" s="12" t="n"/>
+      <c r="I96" s="12" t="n"/>
+      <c r="J96" s="12" t="n"/>
+      <c r="K96" s="12" t="n"/>
+      <c r="L96" s="12" t="n"/>
+      <c r="M96" s="12" t="n"/>
+    </row>
+    <row r="97">
+      <c r="C97" s="11" t="inlineStr">
+        <is>
+          <t>MÍNIMO</t>
+        </is>
+      </c>
+      <c r="D97" s="10">
+        <f>MIN(D3:D90)</f>
         <v/>
       </c>
-      <c r="E96" s="10">
-        <f>MAX(E3:E91)</f>
+      <c r="E97" s="10">
+        <f>MIN(E3:E90)</f>
         <v/>
       </c>
-      <c r="F96" s="10">
-        <f>MAX(F3:F91)</f>
+      <c r="F97" s="10">
+        <f>MIN(F3:F90)</f>
         <v/>
       </c>
-      <c r="G96" s="10">
-        <f>MAX(G3:G91)</f>
+      <c r="G97" s="10">
+        <f>MIN(G3:G90)</f>
         <v/>
       </c>
-      <c r="H96" s="10">
-        <f>MAX(H3:H91)</f>
+      <c r="H97" s="10">
+        <f>MIN(H3:H90)</f>
         <v/>
       </c>
-      <c r="I96" s="10">
-        <f>MAX(I3:I91)</f>
+      <c r="I97" s="10">
+        <f>MIN(I3:I90)</f>
         <v/>
       </c>
-      <c r="J96" s="10">
-        <f>MAX(J3:J91)</f>
+      <c r="J97" s="10">
+        <f>MIN(J3:J90)</f>
         <v/>
       </c>
-      <c r="K96" s="10">
-        <f>MAX(K3:K91)</f>
+      <c r="K97" s="10">
+        <f>MIN(K3:K90)</f>
         <v/>
       </c>
-      <c r="L96" s="10">
-        <f>MAX(L3:L91)</f>
+      <c r="L97" s="10">
+        <f>MIN(L3:L90)</f>
         <v/>
       </c>
-      <c r="M96" s="10">
-        <f>MAX(M3:M91)</f>
+      <c r="M97" s="10">
+        <f>MIN(M3:M90)</f>
         <v/>
       </c>
     </row>
-    <row r="97">
-      <c r="C97" s="12" t="n"/>
-      <c r="D97" s="12" t="n"/>
-      <c r="E97" s="12" t="n"/>
-      <c r="F97" s="12" t="n"/>
-      <c r="G97" s="12" t="n"/>
-      <c r="H97" s="12" t="n"/>
-      <c r="I97" s="12" t="n"/>
-      <c r="J97" s="12" t="n"/>
-      <c r="K97" s="12" t="n"/>
-      <c r="L97" s="12" t="n"/>
-      <c r="M97" s="12" t="n"/>
-    </row>
     <row r="98">
-      <c r="C98" s="11" t="inlineStr">
-        <is>
-          <t>MÍNIMO</t>
-        </is>
-      </c>
-      <c r="D98" s="10">
-        <f>MIN(D3:D91)</f>
-        <v/>
-      </c>
-      <c r="E98" s="10">
-        <f>MIN(E3:E91)</f>
-        <v/>
-      </c>
-      <c r="F98" s="10">
-        <f>MIN(F3:F91)</f>
-        <v/>
-      </c>
-      <c r="G98" s="10">
-        <f>MIN(G3:G91)</f>
-        <v/>
-      </c>
-      <c r="H98" s="10">
-        <f>MIN(H3:H91)</f>
-        <v/>
-      </c>
-      <c r="I98" s="10">
-        <f>MIN(I3:I91)</f>
-        <v/>
-      </c>
-      <c r="J98" s="10">
-        <f>MIN(J3:J91)</f>
-        <v/>
-      </c>
-      <c r="K98" s="10">
-        <f>MIN(K3:K91)</f>
-        <v/>
-      </c>
-      <c r="L98" s="10">
-        <f>MIN(L3:L91)</f>
-        <v/>
-      </c>
-      <c r="M98" s="10">
-        <f>MIN(M3:M91)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="99">
-      <c r="C99" s="12" t="n"/>
-      <c r="D99" s="12" t="n"/>
-      <c r="E99" s="12" t="n"/>
-      <c r="F99" s="12" t="n"/>
-      <c r="G99" s="12" t="n"/>
-      <c r="H99" s="12" t="n"/>
-      <c r="I99" s="12" t="n"/>
-      <c r="J99" s="12" t="n"/>
-      <c r="K99" s="12" t="n"/>
-      <c r="L99" s="12" t="n"/>
-      <c r="M99" s="12" t="n"/>
-    </row>
+      <c r="C98" s="12" t="n"/>
+      <c r="D98" s="12" t="n"/>
+      <c r="E98" s="12" t="n"/>
+      <c r="F98" s="12" t="n"/>
+      <c r="G98" s="12" t="n"/>
+      <c r="H98" s="12" t="n"/>
+      <c r="I98" s="12" t="n"/>
+      <c r="J98" s="12" t="n"/>
+      <c r="K98" s="12" t="n"/>
+      <c r="L98" s="12" t="n"/>
+      <c r="M98" s="12" t="n"/>
+    </row>
+    <row r="99"/>
+    <row r="100"/>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="E92:E93"/>
-    <mergeCell ref="K92:K93"/>
-    <mergeCell ref="D96:D97"/>
-    <mergeCell ref="E98:E99"/>
-    <mergeCell ref="G98:G99"/>
-    <mergeCell ref="C94:C95"/>
-    <mergeCell ref="M98:M99"/>
-    <mergeCell ref="K94:K95"/>
-    <mergeCell ref="M94:M95"/>
-    <mergeCell ref="J98:J99"/>
-    <mergeCell ref="L92:L93"/>
-    <mergeCell ref="E94:E95"/>
-    <mergeCell ref="K96:K97"/>
-    <mergeCell ref="H98:H99"/>
-    <mergeCell ref="F94:F95"/>
-    <mergeCell ref="I92:I93"/>
-    <mergeCell ref="H94:H95"/>
-    <mergeCell ref="I96:I97"/>
-    <mergeCell ref="G92:G93"/>
-    <mergeCell ref="K98:K99"/>
-    <mergeCell ref="J94:J95"/>
-    <mergeCell ref="F96:F97"/>
-    <mergeCell ref="L94:L95"/>
-    <mergeCell ref="D92:D93"/>
-    <mergeCell ref="H96:H97"/>
-    <mergeCell ref="I98:I99"/>
-    <mergeCell ref="F92:F93"/>
-    <mergeCell ref="L96:L97"/>
-    <mergeCell ref="G94:G95"/>
-    <mergeCell ref="C96:C97"/>
-    <mergeCell ref="I94:I95"/>
-    <mergeCell ref="J96:J97"/>
-    <mergeCell ref="H92:H93"/>
-    <mergeCell ref="L98:L99"/>
-    <mergeCell ref="D98:D99"/>
-    <mergeCell ref="G96:G97"/>
-    <mergeCell ref="M96:M97"/>
-    <mergeCell ref="F98:F99"/>
-    <mergeCell ref="D94:D95"/>
-    <mergeCell ref="M92:M93"/>
-    <mergeCell ref="J92:J93"/>
-    <mergeCell ref="E96:E97"/>
-    <mergeCell ref="C98:C99"/>
-    <mergeCell ref="C92:C93"/>
+    <mergeCell ref="J93:J94"/>
+    <mergeCell ref="L91:L92"/>
+    <mergeCell ref="I95:I96"/>
+    <mergeCell ref="I91:I92"/>
+    <mergeCell ref="K91:K92"/>
+    <mergeCell ref="L97:L98"/>
+    <mergeCell ref="H93:H94"/>
+    <mergeCell ref="F95:F96"/>
+    <mergeCell ref="C97:C98"/>
+    <mergeCell ref="G97:G98"/>
+    <mergeCell ref="L93:L94"/>
+    <mergeCell ref="I97:I98"/>
+    <mergeCell ref="D95:D96"/>
+    <mergeCell ref="F91:F92"/>
+    <mergeCell ref="J95:J96"/>
+    <mergeCell ref="J91:J92"/>
+    <mergeCell ref="D91:D92"/>
+    <mergeCell ref="C93:C94"/>
+    <mergeCell ref="G93:G94"/>
+    <mergeCell ref="I93:I94"/>
+    <mergeCell ref="D97:D98"/>
+    <mergeCell ref="G95:G96"/>
+    <mergeCell ref="F97:F98"/>
+    <mergeCell ref="F93:F94"/>
+    <mergeCell ref="C95:C96"/>
+    <mergeCell ref="E95:E96"/>
+    <mergeCell ref="M95:M96"/>
+    <mergeCell ref="M91:M92"/>
+    <mergeCell ref="C91:C92"/>
+    <mergeCell ref="E91:E92"/>
+    <mergeCell ref="G91:G92"/>
+    <mergeCell ref="D93:D94"/>
+    <mergeCell ref="E97:E98"/>
+    <mergeCell ref="K97:K98"/>
+    <mergeCell ref="M97:M98"/>
+    <mergeCell ref="M93:M94"/>
+    <mergeCell ref="H95:H96"/>
+    <mergeCell ref="H91:H92"/>
+    <mergeCell ref="L95:L96"/>
+    <mergeCell ref="J97:J98"/>
+    <mergeCell ref="K93:K94"/>
+    <mergeCell ref="E93:E94"/>
+    <mergeCell ref="H97:H98"/>
+    <mergeCell ref="K95:K96"/>
   </mergeCells>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup orientation="portrait" paperSize="9" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Anexo 3: two decimals in the PROMEDIO row
</commit_message>
<xml_diff>
--- a/Anexo_03_Estadisticas_pre_limpieza/Anexo_03_Estadisticas_pre_limpieza.xlsx
+++ b/Anexo_03_Estadisticas_pre_limpieza/Anexo_03_Estadisticas_pre_limpieza.xlsx
@@ -126,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -145,6 +145,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5216,35 +5219,35 @@
         <f>AVERAGE(G3:G90)</f>
         <v/>
       </c>
-      <c r="H91" s="6">
+      <c r="H91" s="8">
         <f>AVERAGE(H3:H90)</f>
         <v/>
       </c>
-      <c r="I91" s="6">
+      <c r="I91" s="8">
         <f>AVERAGE(I3:I90)</f>
         <v/>
       </c>
-      <c r="J91" s="6">
+      <c r="J91" s="8">
         <f>AVERAGE(J3:J90)</f>
         <v/>
       </c>
-      <c r="K91" s="6">
+      <c r="K91" s="8">
         <f>AVERAGE(K3:K90)</f>
         <v/>
       </c>
-      <c r="L91" s="6">
+      <c r="L91" s="8">
         <f>AVERAGE(L3:L90)</f>
         <v/>
       </c>
-      <c r="M91" s="6">
+      <c r="M91" s="8">
         <f>AVERAGE(M3:M90)</f>
         <v/>
       </c>
-      <c r="N91" s="6">
+      <c r="N91" s="8">
         <f>AVERAGE(N3:N90)</f>
         <v/>
       </c>
-      <c r="O91" s="6">
+      <c r="O91" s="8">
         <f>AVERAGE(O3:O90)</f>
         <v/>
       </c>

</xml_diff>